<commit_message>
readable HydroRivers database, graph from this database
visualizing not working yet
</commit_message>
<xml_diff>
--- a/graph_data.xlsx
+++ b/graph_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github Repositories\Sensor-Placement-Optimization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE9E7ACE-EC95-40B8-A890-34A9E2179AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86A1E20-CC77-4CCA-BC70-B01E0EB60A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="8844" windowHeight="12360" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3564" windowWidth="12960" windowHeight="7176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dummy_graph_nodes" sheetId="1" r:id="rId1"/>

</xml_diff>